<commit_message>
progress: 74 village workbooks (sivaramans-llin 2026-10-10T22:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Arambakkam_13.528696_80.064099.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Arambakkam_13.528696_80.064099.xlsx
@@ -686,6 +686,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -693,6 +698,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -700,6 +710,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -707,6 +722,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A1, 4A2, 5A1A, 5A1B, 5A1C, 5A2, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -714,6 +734,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2A1, 2A2A1A, 2A2A2, 2A2A3, 2A2A4, 2A2B, 2A2C, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -721,6 +746,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1A, 1B, 29, 2A, 2B, 30, 31, 32, 33A, 33B, 34, 35, 36A, 36B, 37, 38, 39, 3A, 3B, 4, 40, 41, 42, 43, 44, 5A1A1, 5A2, 5B1A1, 5B1A2, 5B1B, 5B2, 5B3A, 5B3B, 5B4, 5B5, 5B6, 5B7, 5B8, 5B9, 6A, 6B, 7, 8A, 8B1, 8B2A, 8B2B, 8C1A, 8C1B1, 8C1B2, 8C1B3, 8C1C, 8C2, 9A1A1A, 9A1A2, 9A1B, 9A2, 9B1A, 9B1B</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -728,6 +758,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A1A, 1A2, 2A1A1A1, 2A1A2, 2A1B, 2A2, 2B1A1, 2B1A2, 2B1B, 2B2, 2B3A1, 2B3A2, 2B3A3A, 2B3B, 2B3C, 2B3D, 3A1A, 3A2, 3A3, 3A4, 3A5, 3B1A, 3B1B, 3B2, 4A, 4B1, 4B2A, 4B2B, 4B2C, 4B3, 4B4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -735,6 +770,11 @@
           <t>266</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -742,6 +782,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -749,6 +794,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -756,6 +806,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -763,6 +818,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10, 11, 115B1A2A, 12A, 12B, 13, 14, 14A, 14B, 15, 15A1A1, 15A1A2, 15A1B1, 15A1B2A, 15A1C, 15A2, 15B, 15B1A1, 15B1B1B, 15B1B2A1, 15B1C, 15B2, 16, 17, 18, 19, 1A1A1, 1A1A2, 1A1B, 1A2A1A, 1A2A2A, 1A2B, 1A3A1, 1A3A2, 1A3B, 1B1, 1B2, 20, 21, 22, 23, 24, 25, 26, 27, 29, 2A1A1A, 2A1B1, 2A2, 2A3, 2A4, 2A5, 2A6, 2B1, 2B2, 30, 31, 32, 33, 34, 35, 36, 38, 39, 3A1A, 3A1B, 3A2, 3B, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 4A1, 4A2, 4A3, 4A4, 4A5, 4A6, 4B, 4C, 4D, 4E, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 5A1, 5A2, 5B1A, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 6A1, 6B1A1A, 70, 71, 72, 73, 74, 75, 76, 77, 7A1A, 7A2, 8, 9A1A, 9A1B</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -770,11 +830,21 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 11A1A1, 11A2, 11B1A, 11B1B1, 11B1B2, 11B2A1, 11B2B, 12A1, 12B, 12C, 12D, 12E, 13A1A1, 13B, 14A1A, 14A2, 14B, 15, 16A, 16B, 16C, 17A, 17B, 18A1A, 18A2, 18B, 19A1A, 19A1B, 19B1A, 19B2, 2, 20, 21, 22A1, 22B, 23A1, 23A2, 23B, 24, 25A1A1, 25A1B, 25A2, 25B, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 37, 38, 39, 40, 41, 42, 43, 44, 4A, 4B, 4C, 4D, 5, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 7, 8, 9A, 9B, 9C, 9D, 9E, 9F</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
           <t>278</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B1A1, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 2A1A1, 2A1A2A, 2A1B, 2A1C, 2A2A1, 2A2B, 2B, 3A1, 3A2, 3A3, 3A4, 3B, 4, 49, 5, 6, 7A1, 7A2, 7B, 8A, 8B1, 8B2, 8C1, 8C2, 8D1, 8D2, 9A1, 9A2, 9B1, 9B2, 9C1A, 9C1B, 9C2, 9C3A1, 9C3B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 82 village workbooks (sivaramans-llin 2026-10-11T13:05:01Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Arambakkam_13.528696_80.064099.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Arambakkam_13.528696_80.064099.xlsx
@@ -854,6 +854,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2A, 10A2B, 10A2C, 10B1, 10B2, 10C, 11, 12, 13, 14, 15, 16, 2, 3, 4A, 4B1A1, 4B1B, 4B2, 4B3, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -861,6 +866,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B1, 2B2, 2C1, 2C2, 3A1, 3A2, 3B1, 3B2, 3C1, 3C2, 3D, 3E1, 3E2, 3F, 3G1, 3G2</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -868,6 +878,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -875,6 +890,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -882,6 +902,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -889,6 +914,11 @@
           <t>288</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -896,6 +926,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A1, 11A2, 11B, 12A1A1, 12A1A2, 12A1A3, 12A1A4, 12A1A5, 12A1A6, 12A1A7, 12A1B, 12A2, 12B1A, 12B1B, 12B2, 13A1, 13A2, 13B, 14A1, 14A2, 14A3, 14B1, 14B2, 14B3, 14C1A, 14C1B, 14C2A, 14C2B, 15, 16A1A, 16A1B, 16A2, 16B, 17A, 17B1, 17B2A, 17B2B, 18, 2A1A, 2A1B, 2A1C1, 2A1C2, 2A2, 2B1A, 2B2, 2B3, 2C1, 2C2, 3, 4, 5A, 5B, 5C1, 5C2, 5C3, 6A1, 6A2, 6A3, 6B1, 6B2, 7, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -903,6 +938,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 10, 100, 101A, 102, 103, 104, 105, 106, 107, 108, 109, 11, 110, 111, 112, 113, 114, 115, 116, 117, 118, 119, 12, 120, 121, 13, 14A, 14B, 15A, 15B, 16, 17, 18A1, 18A1A1A1A1, 18A1A1B, 18A2, 18A3, 18C, 19A, 19B, 19C1A, 19E, 20A, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 5A1A, 5B, 5C, 5D, 5E, 5F, 5G, 60, 61, 62, 63, 64A, 64B, 65, 66, 67, 68, 69, 6A1A, 6B, 6C, 6D, 6E, 6F, 6G, 6H, 6I, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 7A, 7B, 7C, 7D, 7E, 7F, 7G, 7H, 7J, 7K, 7L, 7M, 7N, 8, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 9A, 9B, 9C, 9D, 9E, 9F, 9G</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -910,6 +950,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -917,6 +962,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -924,6 +974,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -931,6 +986,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B1, 1B2A1A1A, 1B2B, 1B3A1A1, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 3A1, 3A2, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -938,6 +998,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 1A1A1A1A1, 1A1B, 1A1C, 1A1D, 1A1E, 1A2, 1B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2A1B, 2A2, 2A3, 2A4, 2A5, 2A6, 2B, 2C, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A1A1A, 3B, 3C1, 3C2, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 4A1A, 4B, 50, 51, 52, 53, 54, 55, 5A1A1, 5A1B, 5A2, 5A3, 5A4, 5A5, 5A6, 5A7, 5A8, 5A9, 5B, 6A, 6B1A, 6B1A2, 6B2, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -945,6 +1010,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B1, 2B2A1, 2C1A, 2C1A1A, 2C1C, 2C2, 2C3, 2C4, 2C5, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A1A, 3A2, 3B, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -952,6 +1022,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -959,6 +1034,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -966,6 +1046,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12A, 12B, 13A, 13B, 14A1, 14A2, 14B, 1A, 1B, 1C, 1D, 2A, 2B, 2C, 2D, 2E, 2F1, 2F2, 2G, 3, 4A, 4B, 4C1, 4C2, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -973,6 +1058,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 12A, 12B, 2A, 2B1, 2B2, 2B3, 2C, 2D, 2E, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -980,6 +1070,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1A1A, 12A1A2, 12A1A3, 12A1B, 12A1C, 12A2, 12B1A, 12B1B, 12B2, 17, 2A, 2B, 3, 4, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 5H, 5I, 6A1A, 6A1B, 6A2, 6B, 6C, 7A1, 7B, 7C, 7D, 7E, 7F, 7G, 7H, 7I, 7J, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -987,6 +1082,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4A, 4B, 4C, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -994,6 +1094,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1001,6 +1106,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1008,6 +1118,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1015,6 +1130,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1022,6 +1142,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1029,6 +1154,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1036,6 +1166,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1043,6 +1178,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1050,6 +1190,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1057,6 +1202,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1064,6 +1214,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2A, 1B2B1, 1B2B2, 1B2B3, 2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1071,6 +1226,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1078,6 +1238,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A1A1, 1A1B, 1A2, 1A3, 1A4A1A1, 1A4B, 1A4C, 1A4D, 1B, 2, 3, 4, 5A, 5B, 6A, 6B1, 6B2, 6B3, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1085,6 +1250,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1092,6 +1262,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1099,6 +1274,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1106,6 +1286,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1113,6 +1298,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1120,6 +1310,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A1B, 1A2A, 1A2B, 1B1, 1B2A, 1B2B, 1C, 1D, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B1A1, 2B2, 2B3, 2B4, 2B5, 30, 31, 32, 33, 34, 35, 36, 37, 38, 3A, 3B, 5A1A1A, 5A1A1B1, 5A2A, 5A2B, 5B1, 5B2, 6A, 6B, 6C1A1A1, 6C1B, 6C2, 6D1A1, 6D1A2, 6D1A3, 6D1B1, 6D1C, 6D2, 6E1A, 6E1B, 6E1C, 6E1D, 6E1E, 6E1F, 6E2, 7A1A1A1, 7A1A2, 7A1B1, 7A1C1, 7A1C2, 7A1D, 7A1E, 7A2A, 7A2B, 7B, 8A1, 8A2, 8A3, 8B1A1, 8B1A2, 8B1B, 8B1C, 8B1D, 8B2A1A1, 8B2A2, 8B2A3, 8B2B1, 8B2B2, 9A1A1, 9A2, 9B1, 9B2, 9B3</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1127,6 +1322,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>10, 11A1, 11A2, 11B, 12, 13, 14, 15, 16, 17, 18A, 18B, 19, 1A1A1A, 1A1A2, 1A1B1, 1A1C, 1A2, 1B1, 1B2, 1B3, 1B4, 1B5A, 1B5B, 1B6A, 1B6B, 1B7, 2, 20, 21, 22, 23, 24, 25, 26, 3A1A1, 3A1B, 3A1C, 3A2, 3B, 4A1A, 4A1B, 4A2, 4B, 4C1, 4C2, 5, 6A1A1A, 6A1B, 6A2A, 6A2B, 6B1A, 6B1B, 6B2, 6C1, 6C2, 7, 8A1, 8A2A, 8A2B, 8B1, 8B2, 8B3, 8B4, 8B5, 8B6, 8B7, 8B8, 8C, 8D1, 8D2A, 8D2B, 8D3, 8D4, 8D5, 8D6, 8D7, 8E1, 8E2, 8E4, 8E5, 8E6, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1134,6 +1334,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1141,6 +1346,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13A, 13B1, 13B2, 14, 15, 16, 17, 18, 19A, 19B, 1A, 1B1A, 1B1B, 1B2, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39A, 39B, 39C, 39D, 3A1A1, 3A1A2, 3A1A3, 3A1B, 3A2, 3A3, 3A4, 3D, 4, 40, 41, 42, 43, 44A, 44B, 45, 46, 47, 48, 49, 50, 5A, 5B, 61, 62, 63, 6A, 6B, 6C, 7A1A1, 7B, 7C1A1, 7C1B, 7C2, 7D1, 7D2, 7E, 7F, 7G1, 7G2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1148,6 +1358,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1155,6 +1370,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1162,6 +1382,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1169,6 +1394,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C, 3, 4, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1176,6 +1406,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1183,6 +1418,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1190,6 +1430,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1197,6 +1442,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1204,6 +1454,11 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1211,6 +1466,11 @@
           <t>378</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2B, 2C, 2D, 3A, 3B, 4A1A1, 4B, 4C, 4D, 4E, 4F, 4G, 4H, 4J, 5</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1218,6 +1478,11 @@
           <t>381</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1225,6 +1490,11 @@
           <t>385</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 1A, 1B, 2, 3A, 3B, 4A, 4B, 4C, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1232,6 +1502,11 @@
           <t>387</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10A1, 10A2, 10B1, 10B2, 1A1, 1A2, 1B, 2A1A, 2A1B, 2A2, 2B, 3A, 3B, 3C, 4, 5A, 5B, 6, 7A, 7B, 8, 9A, 9B1, 9B2, 9E</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1239,6 +1514,11 @@
           <t>388</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13A, 13B, 13C, 14A1, 14A2, 14B1, 14B2, 15A1, 15A2, 15B1, 15B2, 16A, 16B, 17, 18A, 18B, 19, 2, 20A1, 20A2, 20B, 21, 3, 4, 5A, 5B, 6, 7, 8A, 8B, 9A1, 9A2, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1246,6 +1526,11 @@
           <t>390</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 12A, 12B, 13, 14, 15, 16, 17A, 17B, 18, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1253,6 +1538,11 @@
           <t>393</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1260,6 +1550,11 @@
           <t>397</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16A1, 16A2, 16B, 17, 18, 1A1, 1A2, 1A3, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1267,6 +1562,11 @@
           <t>398</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 13A, 13B, 14A, 14B, 15, 2, 3A, 3B, 4, 5A, 5B, 6, 7, 8A, 8B, 8C, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1274,6 +1574,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 20A, 20B, 21, 2A1, 2A2, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1281,6 +1586,11 @@
           <t>401</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1288,6 +1598,11 @@
           <t>402</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4A1, 4A2, 4B, 5, 6A1, 6A2, 6B, 7A1, 7A2, 7A3, 7B1, 7B2, 7B3, 8, 9A, 9B1, 9B2, 9B3A, 9B3B, 9B4A, 9B4B</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1295,6 +1610,11 @@
           <t>403</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1302,6 +1622,11 @@
           <t>404</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1, 11A2, 11B, 11C, 12A, 12B, 13, 14, 2A1A, 2A1B, 2A2, 2B, 3A1, 3A2, 3B, 3C, 3D, 3E, 3F, 4, 5, 6, 7, 8, 9A, 9B1A1, 9B1B, 9B2, 9C1, 9C2, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1309,6 +1634,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 1A, 1B, 2A1, 2A2, 2B, 3A, 3B, 4A1, 4A2, 4B, 5A, 5B, 6, 7A, 7B, 7C, 7D, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1316,6 +1646,11 @@
           <t>407</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1323,6 +1658,11 @@
           <t>408</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 10E, 10F, 10G, 10H, 10I, 10J, 10K, 10L, 11A1, 11A2, 11B, 12, 13, 14, 2, 3A, 3B, 3C, 4, 5A1A, 5A1B, 5A1C, 5A2, 5B, 6A, 6B, 6C, 7A1, 7A2, 7A3, 7A4, 7A5, 7A6, 7A7, 7B1, 7B10, 7B11, 7B2, 7B3, 7B4, 7B5, 7B6, 7B7, 7B8, 7B9, 7C10, 7C11, 7C12, 7C1A, 7C2, 7C3, 7C4, 7C5, 7C6, 7C7, 7C8, 7C9, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1330,6 +1670,11 @@
           <t>409</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 12A1, 12A2, 12B, 13, 14A1A, 14A2, 14B, 14C, 15, 16, 17, 18, 19, 1A1A2, 2, 3, 4, 5A, 5B1, 5B2, 5C, 5D, 6, 7A, 7B, 7C, 7D1, 7D2, 7E, 8, 9A1, 9A2, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1337,6 +1682,11 @@
           <t>410</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1344,6 +1694,11 @@
           <t>413</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 10, 13, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6A1, 6A2A1, 6A2A2, 6A2B, 6A2C, 6B1A1A, 6B1A1B, 6B1A2, 6B1B, 6B2A1A, 6B2B, 6B2C, 6B3, 6B4A1A1, 6B4B, 6B5A1, 7, 8A1, 8A2, 8B1A1, 8B1B, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1351,6 +1706,11 @@
           <t>415</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 12, 13A, 13B, 13C, 14A, 14B, 15A, 15B, 15C, 16, 17, 18, 19, 2, 20, 21, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1358,6 +1718,11 @@
           <t>416</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1C, 1D, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1365,6 +1730,11 @@
           <t>417</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1372,6 +1742,11 @@
           <t>418</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C, 3D, 3E, 3F1, 3F2, 3G1A, 3G1A2, 3G1B, 3G2, 3G3, 3H, 3J, 3K, 3L, 3M, 3N, 4A1, 4A2, 4B, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1379,6 +1754,11 @@
           <t>421</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1386,6 +1766,11 @@
           <t>422</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1393,6 +1778,11 @@
           <t>424</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1400,6 +1790,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2, 3A1A1, 3A1A2, 3A1A3, 3A1A4, 3A1B, 3A2, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1407,6 +1802,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C1, 3</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1414,6 +1814,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1421,6 +1826,11 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1428,6 +1838,11 @@
           <t>434</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1435,6 +1850,11 @@
           <t>436</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10, 100, 101, 102, 103, 104, 105, 106, 107, 108, 109, 11, 110, 111, 112, 113, 114, 115, 116, 117, 118, 119, 12, 120, 121, 122, 123, 13, 14, 15, 16, 17, 18, 19, 1A1A1, 1A1A2, 1A1A3, 1A1A4, 1A1B, 1A2, 1A3, 1B, 1C, 1D, 1E, 1F, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A, 3B, 3C1, 3C2, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 7, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 8, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1442,6 +1862,11 @@
           <t>437</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1449,6 +1874,11 @@
           <t>440</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1456,6 +1886,11 @@
           <t>441</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1463,6 +1898,11 @@
           <t>445</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1470,6 +1910,11 @@
           <t>446</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1477,6 +1922,11 @@
           <t>447</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1484,6 +1934,11 @@
           <t>448</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1491,6 +1946,11 @@
           <t>452</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 10E, 11A, 11B, 11C, 11D, 2, 3, 4A1, 4A2, 4A3, 4A4, 4B1, 4B2, 5A, 5B, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1498,6 +1958,11 @@
           <t>456</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 3A, 3B, 4, 5A, 5B, 6A, 6B, 7, 8A, 8B, 8C, 8D, 8E, 9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1505,6 +1970,11 @@
           <t>458</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2, 3, 4A, 4B, 4C, 4D, 5A, 5B, 5C, 5D, 5E, 5F, 6A, 6B, 6C, 6D, 6E, 6F</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1512,6 +1982,11 @@
           <t>462</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1519,6 +1994,11 @@
           <t>464</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1526,6 +2006,11 @@
           <t>467</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1533,6 +2018,11 @@
           <t>468</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1540,6 +2030,11 @@
           <t>469</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3A, 3B, 3C, 3D1, 3D2, 4, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 5H, 6, 7A, 7B, 7C, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1547,6 +2042,11 @@
           <t>472</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 3C, 3D, 4, 5A, 5B, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 7A, 7B, 8A, 8B, 8C, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1554,6 +2054,11 @@
           <t>473</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1A, 1B1A1, 1B1A2, 1B1B, 1B2, 1B3, 2A1A, 2A1B, 2A1C, 2A2A, 2A2B1, 2A2B2, 2B1A1, 2B1A2, 2B1B1, 2B1B2, 2B2, 2B3, 3, 4, 5, 6, 7A, 7B, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1561,6 +2066,11 @@
           <t>476</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 11, 1A, 1B, 2A1, 2A2, 2A3, 2A4, 2B1, 2B2A, 2B2B, 3, 4, 5, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1568,6 +2078,11 @@
           <t>478</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B1, 10B2, 11A, 11B, 12A1A, 12B, 12C1, 12C2, 12D, 13A1A, 13B, 13C1, 13C2, 13D, 14, 15A, 15B, 16, 2, 3, 4, 5, 6A, 6B, 7, 8A, 8B, 9A1, 9A2, 9B1, 9B2, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1575,6 +2090,11 @@
           <t>482</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 4A, 4B, 4C, 4D, 5A1, 5A2, 5A3, 5A4, 5A5, 5A6, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1582,6 +2102,11 @@
           <t>483</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1589,6 +2114,11 @@
           <t>492</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1596,6 +2126,11 @@
           <t>493</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>10, 1A1A, 1A1B, 1A1C, 1A1D, 1A2, 1B, 2A, 2B, 2C1, 2C2, 3, 4, 5, 6A, 6B, 7, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1603,11 +2138,21 @@
           <t>496</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 3, 4A1A, 4A1B, 4A2, 4B, 5A, 5B, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
           <t>563</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>